<commit_message>
feat(masterdata): add StatusEffect Luban table (haste row) [Phase 3c]
source/StatusEffect.xlsx + convert registration -> Datas/#StatusEffect.xlsx
and __tables__ entry. int `id` index (matches core int EffectId, industry
standard per lop-repo-topology key convention), string enum columns +
inline single modifier (project convention). One haste row (MoveSpeed
+30% PercentAdd, 100 ticks) for verification.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__tables__.xlsx
+++ b/table/Datas/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,6 +682,47 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TbStatusEffect</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>StatusEffect</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>#StatusEffect.xlsx</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>StatusEffect</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(masterdata): add Ability Luban table (haste row) [Phase 3e]
source/Ability.xlsx + convert registration -> Datas/#Ability.xlsx and
__tables__ entry. int `id` PK + string `code` alias (key convention).
One haste ability row (id 1, code "haste", produces effect 1).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__tables__.xlsx
+++ b/table/Datas/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -723,6 +723,47 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TbAbility</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ability</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>#Ability.xlsx</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ability</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(masterdata): TbAction 테이블 은퇴 — source/Action.xlsx·#Action.xlsx 삭제 + convert에서 Action 제외 (slice 5)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__tables__.xlsx
+++ b/table/Datas/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -604,12 +604,12 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TbAction</t>
+          <t>TbItem</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>#Action.xlsx</t>
+          <t>#Item.xlsx</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -635,7 +635,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -645,12 +645,12 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TbItem</t>
+          <t>TbStatusEffect</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>StatusEffect</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>#Item.xlsx</t>
+          <t>#StatusEffect.xlsx</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>id</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -676,7 +676,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>StatusEffect</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -686,12 +686,12 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TbStatusEffect</t>
+          <t>TbAbility</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>StatusEffect</t>
+          <t>Ability</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>#StatusEffect.xlsx</t>
+          <t>#Ability.xlsx</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -717,52 +717,11 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>StatusEffect</t>
+          <t>Ability</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>TbAbility</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Ability</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>#Ability.xlsx</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Ability</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(masterdata): TbCombatConfig 전역 전투 튜닝 테이블(서버 group s) 저작
</commit_message>
<xml_diff>
--- a/table/Datas/__tables__.xlsx
+++ b/table/Datas/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,7 +474,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>TbCharacter</t>
@@ -505,17 +504,13 @@
           <t>map</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Character</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>TbSkin</t>
@@ -546,17 +541,13 @@
           <t>map</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Skin</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>TbSkinAsset</t>
@@ -597,11 +588,8 @@
           <t>SkinAsset</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>TbItem</t>
@@ -632,17 +620,13 @@
           <t>map</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>TbStatusEffect</t>
@@ -673,17 +657,13 @@
           <t>map</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>StatusEffect</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>TbAbility</t>
@@ -714,14 +694,53 @@
           <t>map</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>Ability</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TbCombatConfig</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CombatConfig</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>#CombatConfig.xlsx</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>CombatConfig(전역 전투 튜닝, 서버 전용)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(masterdata): TbStatusEffectView — 상태이상 id → 이펙트 주소
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__tables__.xlsx
+++ b/table/Datas/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,7 +780,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>TbAbilityView</t>
@@ -821,8 +820,51 @@
           <t>AbilityView</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TbStatusEffectView</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>StatusEffectView</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>#StatusEffectView.xlsx</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>StatusEffectView</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(masterdata): GameMode/Map/Queue 테이블 신설 + matchmaking 타깃 추가
매치메이킹 마스터데이터를 Luban 단일 진실원본으로 통합. 매칭 서버 전용
비기본 그룹 m을 만들어 3개 테이블만 typescript-json + json으로 뽑는다.
기존 sub_game_data XML 5종을 값 그대로 이관(전부 min 2 / max 8) — 동작 무변화.

TbMap의 value_type을 'Map'이 아닌 'GameMap'으로 등록했다 — 'Map'은
typescript-json 타깃 생성 코드에서 전역 Map<K,V> 제네릭 타입과 이름이
충돌해 tsc 빌드가 깨진다(TS2315/TS2558). 테이블 stem(tbmap)과
Tables.TbMap 접근자는 full_name 기준이라 영향 없음.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__tables__.xlsx
+++ b/table/Datas/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -822,7 +822,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>TbStatusEffectView</t>
@@ -863,8 +862,126 @@
           <t>StatusEffectView</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TbGameMode</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>GameMode</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>#GameMode.xlsx</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>c,s,m</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>GameMode</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TbMap</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GameMap</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>#Map.xlsx</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>c,s,m</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>GameMap</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TbQueue</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Queue</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>#Queue.xlsx</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>c,s,m</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Queue</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(masterdata): Flappy Race 튜닝 테이블을 추가한다
새 전진·플랩·중력·몸 규격·반발계수를 기획이 엑셀로 조정한다. group을 비워
클·서 양쪽 패키지에 생성되게 했다 — 클라 예측이 서버와 같은 값을 써야 한다.
</commit_message>
<xml_diff>
--- a/table/Datas/__tables__.xlsx
+++ b/table/Datas/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -983,6 +983,41 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TbFlappyConfig</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FlappyConfig</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>#FlappyConfig.xlsx</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>FlappyConfig(Flappy Race 튜닝, 클·서 공용)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>